<commit_message>
chore(demo): offline demo script and 10-rule dirty fixtures
demo.sh: 서버 기동→clean/dirty 검수→report.md(오프라인). dirty 샘플을 10개 룰 각 1건씩 유발하도록 재설계(csv+xlsx).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/dirty/inventory.xlsx
+++ b/data/samples/dirty/inventory.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,16 +444,20 @@
           <t>SKU-1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>10</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>8</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -462,16 +466,20 @@
           <t>SKU-2</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>10</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>8</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -480,34 +488,108 @@
           <t>SKU-3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>10</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>8</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>SKU-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SKU-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SKU-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>SKU-9</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>